<commit_message>
Update packing list weights: 0.5 kg/EA, N.W. 1.0 kg
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JjYpiojBAR1VpedMN3mqRJ
</commit_message>
<xml_diff>
--- a/수출서류/JJWORLDTRADE_PO2026101501_Invoice_PackingList.xlsx
+++ b/수출서류/JJWORLDTRADE_PO2026101501_Invoice_PackingList.xlsx
@@ -34,7 +34,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">N.W. = 1.0 kg/EA x 2 EA (per CEO)</t>
+          <t xml:space="preserve">N.W. = 0.5 kg/EA x 2 EA (per CEO)</t>
         </r>
       </text>
     </comment>
@@ -46,7 +46,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">G.W. estimate incl. carton/packing - confirm by actual weighing</t>
+          <t xml:space="preserve">G.W. estimate incl. carton/packing (+0.5 kg) - confirm by actual weighing</t>
         </r>
       </text>
     </comment>
@@ -374,11 +374,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -423,11 +427,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -702,379 +706,379 @@
   <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="4" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="5"/>
+      <c r="G4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="5"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="4" t="s">
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="5"/>
+      <c r="G5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="4" t="s">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="5"/>
+      <c r="G6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="5"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="4" t="s">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="5" t="s">
+      <c r="F7" s="5"/>
+      <c r="G7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="5"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2" t="s">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3" t="s">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3" t="s">
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="5" t="s">
+      <c r="B18" s="5"/>
+      <c r="C18" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="4" t="s">
+      <c r="D18" s="6"/>
+      <c r="E18" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="G18" s="5" t="s">
+      <c r="F18" s="5"/>
+      <c r="G18" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="5" t="s">
+      <c r="B19" s="5"/>
+      <c r="C19" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="4" t="s">
+      <c r="D19" s="6"/>
+      <c r="E19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="5" t="s">
+      <c r="F19" s="5"/>
+      <c r="G19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="5" t="s">
+      <c r="B20" s="5"/>
+      <c r="C20" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="4" t="s">
+      <c r="D20" s="6"/>
+      <c r="E20" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="5" t="s">
+      <c r="F20" s="5"/>
+      <c r="G20" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="H20" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="5" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E23" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G23" s="7" t="n">
+      <c r="G23" s="8" t="n">
         <v>1000</v>
       </c>
-      <c r="H23" s="7" t="n">
+      <c r="H23" s="8" t="n">
         <f aca="false">E23*G23</f>
         <v>2000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="9" t="n">
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="10" t="n">
         <f aca="false">SUM(E23:E23)</f>
         <v>2</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="G24" s="9"/>
-      <c r="H24" s="10" t="n">
+      <c r="G24" s="10"/>
+      <c r="H24" s="11" t="n">
         <f aca="false">SUM(H23:H23)</f>
         <v>2000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E30" s="12" t="s">
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E30" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E33" s="13" t="s">
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E33" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E34" s="13" t="s">
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E34" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="45">
@@ -1142,394 +1146,394 @@
   <dimension ref="A1:H36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="4" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="5"/>
+      <c r="G4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="5"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="4" t="s">
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="5"/>
+      <c r="G5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="5"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="4" t="s">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="5"/>
+      <c r="G6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="5"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="4" t="s">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="5" t="s">
+      <c r="F7" s="5"/>
+      <c r="G7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="5"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2" t="s">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3" t="s">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3" t="s">
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="5" t="s">
+      <c r="B18" s="5"/>
+      <c r="C18" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="4" t="s">
+      <c r="D18" s="6"/>
+      <c r="E18" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="G18" s="5" t="s">
+      <c r="F18" s="5"/>
+      <c r="G18" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="5" t="s">
+      <c r="B19" s="5"/>
+      <c r="C19" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="4" t="s">
+      <c r="D19" s="6"/>
+      <c r="E19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="5" t="s">
+      <c r="F19" s="5"/>
+      <c r="G19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H19" s="5"/>
+      <c r="H19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="5" t="s">
+      <c r="B20" s="5"/>
+      <c r="C20" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="4" t="s">
+      <c r="D20" s="6"/>
+      <c r="E20" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="5" t="s">
+      <c r="F20" s="5"/>
+      <c r="G20" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="H20" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="5" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="14" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G23" s="15" t="n">
+      <c r="E23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G23" s="16" t="n">
         <f aca="false">ROUND(21*14*14/1000000,4)</f>
         <v>0.0041</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="H23" s="7" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9" t="n">
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="10" t="n">
         <f aca="false">SUM(D23:D23)</f>
         <v>2</v>
       </c>
-      <c r="E24" s="16" t="n">
+      <c r="E24" s="17" t="n">
         <f aca="false">SUM(E23:E23)</f>
-        <v>2</v>
-      </c>
-      <c r="F24" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="17" t="n">
         <f aca="false">SUM(F23:F23)</f>
-        <v>2.5</v>
-      </c>
-      <c r="G24" s="17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G24" s="18" t="n">
         <f aca="false">SUM(G23:G23)</f>
         <v>0.0041</v>
       </c>
-      <c r="H24" s="9"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
+      <c r="H24" s="10"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E32" s="12" t="s">
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E32" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E35" s="13" t="s">
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E35" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E36" s="13" t="s">
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E36" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="46">

</xml_diff>

<commit_message>
Set actual weights: N.W. 0.4 kg (0.2 kg/EA), G.W. 0.7 kg
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JjYpiojBAR1VpedMN3mqRJ
</commit_message>
<xml_diff>
--- a/수출서류/JJWORLDTRADE_PO2026101501_Invoice_PackingList.xlsx
+++ b/수출서류/JJWORLDTRADE_PO2026101501_Invoice_PackingList.xlsx
@@ -34,7 +34,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">N.W. = 0.5 kg/EA x 2 EA (per CEO)</t>
+          <t xml:space="preserve">N.W. = 0.2 kg/EA x 2 EA (per CEO)</t>
         </r>
       </text>
     </comment>
@@ -46,7 +46,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">G.W. estimate incl. carton/packing (+0.5 kg) - confirm by actual weighing</t>
+          <t xml:space="preserve">G.W. incl. packing, actual weight per CEO</t>
         </r>
       </text>
     </comment>
@@ -1430,10 +1430,10 @@
         <v>2</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>1.5</v>
+        <v>0.7</v>
       </c>
       <c r="G23" s="16" t="n">
         <f aca="false">ROUND(21*14*14/1000000,4)</f>
@@ -1455,11 +1455,11 @@
       </c>
       <c r="E24" s="17" t="n">
         <f aca="false">SUM(E23:E23)</f>
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="F24" s="17" t="n">
         <f aca="false">SUM(F23:F23)</f>
-        <v>1.5</v>
+        <v>0.7</v>
       </c>
       <c r="G24" s="18" t="n">
         <f aca="false">SUM(G23:G23)</f>

</xml_diff>